<commit_message>
feat: add fecha_recojo field across all pages, exports and Excel template
- agregar.html: new 'Fecha de Recojo' date input, auto-syncs with emission date
- vales.html: recojo column in table, edit modal, CSV export, WhatsApp template
- diario.html: recojo column in table (13 cols), CSV export
- cobranza.html: recojo in modal table rows and WhatsApp breakdown
- index.html: recojo sub-line in ultimos vales table
- importexport.html: reads FECHA_RECOJO/RECOJO column from CSV import
- js/db.js: fecha_recojo saved to IndexedDB and synced to Supabase
- js/sidebar.js: inline SQL DDL updated with fecha_recojo DATE column
- supabase_setup.sql: fecha_recojo DATE column added (CREATE + ALTER IF NOT EXISTS)
- servidor.py: payload validator normalises fecha_recojo per vale
- crear_excel_grifo.py: Sheet1 now has 15 cols (A-O) with FECHA RECOJO as col C
- Control_Vales_y_Combustible_Grifo.xlsx: regenerated with FECHA RECOJO column
- tanques.html: XSS-safe data-producto on adjustment buttons
</commit_message>
<xml_diff>
--- a/Control_Vales_y_Combustible_Grifo.xlsx
+++ b/Control_Vales_y_Combustible_Grifo.xlsx
@@ -576,23 +576,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -632,23 +633,23 @@
     </row>
     <row r="4">
       <c r="B4" s="3">
-        <f>COUNTA(D8:D100)</f>
+        <f>COUNTA(E8:E100)</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>SUMIFS(I8:I100, H8:H100, "DIESEL B5", M8:M100, "&lt;&gt;ANULADO")</f>
+        <f>SUMIFS(J8:J100, I8:I100, "DIESEL B5", N8:N100, "&lt;&gt;ANULADO")</f>
         <v/>
       </c>
       <c r="H4" s="4">
-        <f>SUMIFS(I8:I100, H8:H100, "PREMIUM", M8:M100, "&lt;&gt;ANULADO")</f>
+        <f>SUMIFS(J8:J100, I8:I100, "PREMIUM", N8:N100, "&lt;&gt;ANULADO")</f>
         <v/>
       </c>
       <c r="K4" s="5">
-        <f>SUMIF(M8:M100, "&lt;&gt;ANULADO", K8:K100)</f>
+        <f>SUMIF(N8:N100, "&lt;&gt;ANULADO", L8:L100)</f>
         <v/>
       </c>
       <c r="M4" s="6">
-        <f>COUNTIF(M8:M100, "ANULADO")</f>
+        <f>COUNTIF(N8:N100, "ANULADO")</f>
         <v/>
       </c>
     </row>
@@ -662,65 +663,70 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>FECHA</t>
+          <t>FECHA EMISIÓN</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
+          <t>FECHA RECOJO</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
           <t>TURNO</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>N° VALE</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>CLIENTE / EMPRESA</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>CONDUCTOR</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>PRODUCTO</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>CANTIDAD (GLN)</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>PRECIO (S/)</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
         <is>
           <t>TOTAL (S/)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr">
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>GRIFERO / ISLA</t>
         </is>
       </c>
-      <c r="M7" s="7" t="inlineStr">
+      <c r="N7" s="7" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
+      <c r="O7" s="7" t="inlineStr">
         <is>
           <t>N° FACTURA / DOC</t>
         </is>
@@ -737,53 +743,58 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="E8" s="8" t="n">
         <v>377</v>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>Transportes Andina S.A.C.</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>A1B-823</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Carlos Rojas</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I8" s="10" t="n">
+      <c r="J8" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="K8" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K8" s="11">
-        <f>I8*J8</f>
-        <v/>
-      </c>
-      <c r="L8" s="8" t="inlineStr">
+      <c r="L8" s="11">
+        <f>J8*K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>Juan P.</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>FACTURADO</t>
         </is>
       </c>
-      <c r="N8" s="8" t="inlineStr">
+      <c r="O8" s="8" t="inlineStr">
         <is>
           <t>F001-00452</t>
         </is>
@@ -800,53 +811,58 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="E9" s="8" t="n">
         <v>378</v>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Constructora del Sur</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>C4F-912</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>Manuel Vega</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I9" s="10" t="n">
+      <c r="J9" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="11" t="n">
+      <c r="K9" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K9" s="11">
-        <f>I9*J9</f>
-        <v/>
-      </c>
-      <c r="L9" s="8" t="inlineStr">
+      <c r="L9" s="11">
+        <f>J9*K9</f>
+        <v/>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
         <is>
           <t>Juan P.</t>
         </is>
       </c>
-      <c r="M9" s="8" t="inlineStr">
+      <c r="N9" s="8" t="inlineStr">
         <is>
           <t>FACTURADO</t>
         </is>
       </c>
-      <c r="N9" s="8" t="inlineStr">
+      <c r="O9" s="8" t="inlineStr">
         <is>
           <t>F001-00455</t>
         </is>
@@ -863,53 +879,58 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="E10" s="12" t="n">
         <v>379</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="n">
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="15" t="n">
+      <c r="K10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="15">
-        <f>I10*J10</f>
-        <v/>
-      </c>
-      <c r="L10" s="12" t="inlineStr">
+      <c r="L10" s="15">
+        <f>J10*K10</f>
+        <v/>
+      </c>
+      <c r="M10" s="12" t="inlineStr">
         <is>
           <t>Pedro M.</t>
         </is>
       </c>
-      <c r="M10" s="12" t="inlineStr">
+      <c r="N10" s="12" t="inlineStr">
         <is>
           <t>ANULADO</t>
         </is>
       </c>
-      <c r="N10" s="12" t="inlineStr">
+      <c r="O10" s="12" t="inlineStr">
         <is>
           <t>ERROR LLENADO</t>
         </is>
@@ -926,53 +947,58 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="E11" s="8" t="n">
         <v>380</v>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>Distribuidora Lima</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>T6U-711</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Jorge Quispe</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>DIESEL B5</t>
         </is>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="J11" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="J11" s="11" t="n">
+      <c r="K11" s="11" t="n">
         <v>16.8</v>
       </c>
-      <c r="K11" s="11">
-        <f>I11*J11</f>
-        <v/>
-      </c>
-      <c r="L11" s="8" t="inlineStr">
+      <c r="L11" s="11">
+        <f>J11*K11</f>
+        <v/>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
         <is>
           <t>Luis G.</t>
         </is>
       </c>
-      <c r="M11" s="8" t="inlineStr">
+      <c r="N11" s="8" t="inlineStr">
         <is>
           <t>FACTURADO</t>
         </is>
       </c>
-      <c r="N11" s="8" t="inlineStr">
+      <c r="O11" s="8" t="inlineStr">
         <is>
           <t>F001-00460</t>
         </is>
@@ -989,53 +1015,58 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="E12" s="8" t="n">
         <v>381</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Transportes Andina S.A.C.</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
         <is>
           <t>A1B-823</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>Carlos Rojas</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I12" s="10" t="n">
+      <c r="J12" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="J12" s="11" t="n">
+      <c r="K12" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K12" s="11">
-        <f>I12*J12</f>
-        <v/>
-      </c>
-      <c r="L12" s="8" t="inlineStr">
+      <c r="L12" s="11">
+        <f>J12*K12</f>
+        <v/>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
         <is>
           <t>Pedro M.</t>
         </is>
       </c>
-      <c r="M12" s="8" t="inlineStr">
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N12" s="8" t="inlineStr">
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1052,53 +1083,58 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="E13" s="8" t="n">
         <v>382</v>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>Minera Horizonte</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>V7X-551</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Alonso Ruiz</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I13" s="10" t="n">
+      <c r="J13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J13" s="11" t="n">
+      <c r="K13" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K13" s="11">
-        <f>I13*J13</f>
-        <v/>
-      </c>
-      <c r="L13" s="8" t="inlineStr">
+      <c r="L13" s="11">
+        <f>J13*K13</f>
+        <v/>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
         <is>
           <t>Mario S.</t>
         </is>
       </c>
-      <c r="M13" s="8" t="inlineStr">
+      <c r="N13" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N13" s="8" t="inlineStr">
+      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1115,53 +1151,58 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="E14" s="8" t="n">
         <v>383</v>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>Constructora del Sur</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>C4F-912</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Manuel Vega</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I14" s="10" t="n">
+      <c r="J14" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="J14" s="11" t="n">
+      <c r="K14" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K14" s="11">
-        <f>I14*J14</f>
-        <v/>
-      </c>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="L14" s="11">
+        <f>J14*K14</f>
+        <v/>
+      </c>
+      <c r="M14" s="8" t="inlineStr">
         <is>
           <t>Juan P.</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr">
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N14" s="8" t="inlineStr">
+      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1178,53 +1219,58 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="E15" s="8" t="n">
         <v>384</v>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Distribuidora Lima</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>T6U-711</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>Jorge Quispe</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I15" s="10" t="n">
+      <c r="J15" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="J15" s="11" t="n">
+      <c r="K15" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K15" s="11">
-        <f>I15*J15</f>
-        <v/>
-      </c>
-      <c r="L15" s="8" t="inlineStr">
+      <c r="L15" s="11">
+        <f>J15*K15</f>
+        <v/>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
         <is>
           <t>Luis G.</t>
         </is>
       </c>
-      <c r="M15" s="8" t="inlineStr">
+      <c r="N15" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N15" s="8" t="inlineStr">
+      <c r="O15" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1241,53 +1287,58 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="E16" s="8" t="n">
         <v>385</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Agropecuaria San José</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>B8K-102</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>Raúl Castro</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I16" s="10" t="n">
+      <c r="J16" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="J16" s="11" t="n">
+      <c r="K16" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K16" s="11">
-        <f>I16*J16</f>
-        <v/>
-      </c>
-      <c r="L16" s="8" t="inlineStr">
+      <c r="L16" s="11">
+        <f>J16*K16</f>
+        <v/>
+      </c>
+      <c r="M16" s="8" t="inlineStr">
         <is>
           <t>Pedro M.</t>
         </is>
       </c>
-      <c r="M16" s="8" t="inlineStr">
+      <c r="N16" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N16" s="8" t="inlineStr">
+      <c r="O16" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1304,53 +1355,58 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="E17" s="12" t="n">
         <v>386</v>
       </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I17" s="14" t="n">
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="15" t="n">
+      <c r="K17" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="15">
-        <f>I17*J17</f>
-        <v/>
-      </c>
-      <c r="L17" s="12" t="inlineStr">
+      <c r="L17" s="15">
+        <f>J17*K17</f>
+        <v/>
+      </c>
+      <c r="M17" s="12" t="inlineStr">
         <is>
           <t>Juan P.</t>
         </is>
       </c>
-      <c r="M17" s="12" t="inlineStr">
+      <c r="N17" s="12" t="inlineStr">
         <is>
           <t>ANULADO</t>
         </is>
       </c>
-      <c r="N17" s="12" t="inlineStr">
+      <c r="O17" s="12" t="inlineStr">
         <is>
           <t>VALE ROTO</t>
         </is>
@@ -1367,53 +1423,58 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="E18" s="8" t="n">
         <v>387</v>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Distribuidora Lima</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>T6U-711</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>Jorge Quispe</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="I18" s="8" t="inlineStr">
         <is>
           <t>DIESEL B5</t>
         </is>
       </c>
-      <c r="I18" s="10" t="n">
+      <c r="J18" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="J18" s="11" t="n">
+      <c r="K18" s="11" t="n">
         <v>16.8</v>
       </c>
-      <c r="K18" s="11">
-        <f>I18*J18</f>
-        <v/>
-      </c>
-      <c r="L18" s="8" t="inlineStr">
+      <c r="L18" s="11">
+        <f>J18*K18</f>
+        <v/>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
         <is>
           <t>Luis G.</t>
         </is>
       </c>
-      <c r="M18" s="8" t="inlineStr">
+      <c r="N18" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N18" s="8" t="inlineStr">
+      <c r="O18" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1430,53 +1491,58 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="E19" s="8" t="n">
         <v>388</v>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>Transportes Andina S.A.C.</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>A1B-823</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Carlos Rojas</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I19" s="10" t="n">
+      <c r="J19" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="J19" s="11" t="n">
+      <c r="K19" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K19" s="11">
-        <f>I19*J19</f>
-        <v/>
-      </c>
-      <c r="L19" s="8" t="inlineStr">
+      <c r="L19" s="11">
+        <f>J19*K19</f>
+        <v/>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
         <is>
           <t>Pedro M.</t>
         </is>
       </c>
-      <c r="M19" s="8" t="inlineStr">
+      <c r="N19" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N19" s="8" t="inlineStr">
+      <c r="O19" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1493,53 +1559,58 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="E20" s="8" t="n">
         <v>389</v>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>Constructora del Sur</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>C4F-912</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>Manuel Vega</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I20" s="10" t="n">
+      <c r="J20" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="J20" s="11" t="n">
+      <c r="K20" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K20" s="11">
-        <f>I20*J20</f>
-        <v/>
-      </c>
-      <c r="L20" s="8" t="inlineStr">
+      <c r="L20" s="11">
+        <f>J20*K20</f>
+        <v/>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
         <is>
           <t>Juan P.</t>
         </is>
       </c>
-      <c r="M20" s="8" t="inlineStr">
+      <c r="N20" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N20" s="8" t="inlineStr">
+      <c r="O20" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1556,53 +1627,58 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="E21" s="8" t="n">
         <v>390</v>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Agropecuaria San José</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>B8K-102</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>Raúl Castro</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I21" s="10" t="n">
+      <c r="J21" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="J21" s="11" t="n">
+      <c r="K21" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K21" s="11">
-        <f>I21*J21</f>
-        <v/>
-      </c>
-      <c r="L21" s="8" t="inlineStr">
+      <c r="L21" s="11">
+        <f>J21*K21</f>
+        <v/>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
         <is>
           <t>Luis G.</t>
         </is>
       </c>
-      <c r="M21" s="8" t="inlineStr">
+      <c r="N21" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N21" s="8" t="inlineStr">
+      <c r="O21" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1619,53 +1695,58 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="E22" s="8" t="n">
         <v>391</v>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Transportes Andina S.A.C.</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>B3M-442</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>Felipe Díaz</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I22" s="10" t="n">
+      <c r="J22" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="J22" s="11" t="n">
+      <c r="K22" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K22" s="11">
-        <f>I22*J22</f>
-        <v/>
-      </c>
-      <c r="L22" s="8" t="inlineStr">
+      <c r="L22" s="11">
+        <f>J22*K22</f>
+        <v/>
+      </c>
+      <c r="M22" s="8" t="inlineStr">
         <is>
           <t>Pedro M.</t>
         </is>
       </c>
-      <c r="M22" s="8" t="inlineStr">
+      <c r="N22" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N22" s="8" t="inlineStr">
+      <c r="O22" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1682,53 +1763,58 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="D23" s="12" t="n">
+      <c r="E23" s="12" t="n">
         <v>392</v>
       </c>
-      <c r="E23" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H23" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" s="14" t="n">
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J23" s="15" t="n">
+      <c r="K23" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="15">
-        <f>I23*J23</f>
-        <v/>
-      </c>
-      <c r="L23" s="12" t="inlineStr">
+      <c r="L23" s="15">
+        <f>J23*K23</f>
+        <v/>
+      </c>
+      <c r="M23" s="12" t="inlineStr">
         <is>
           <t>Mario S.</t>
         </is>
       </c>
-      <c r="M23" s="12" t="inlineStr">
+      <c r="N23" s="12" t="inlineStr">
         <is>
           <t>ANULADO</t>
         </is>
       </c>
-      <c r="N23" s="12" t="inlineStr">
+      <c r="O23" s="12" t="inlineStr">
         <is>
           <t>CORRELATIVO SALTADO</t>
         </is>
@@ -1745,53 +1831,58 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="D24" s="12" t="n">
+      <c r="E24" s="12" t="n">
         <v>393</v>
       </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="14" t="n">
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="15" t="n">
+      <c r="K24" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="15">
-        <f>I24*J24</f>
-        <v/>
-      </c>
-      <c r="L24" s="12" t="inlineStr">
+      <c r="L24" s="15">
+        <f>J24*K24</f>
+        <v/>
+      </c>
+      <c r="M24" s="12" t="inlineStr">
         <is>
           <t>Mario S.</t>
         </is>
       </c>
-      <c r="M24" s="12" t="inlineStr">
+      <c r="N24" s="12" t="inlineStr">
         <is>
           <t>ANULADO</t>
         </is>
       </c>
-      <c r="N24" s="12" t="inlineStr">
+      <c r="O24" s="12" t="inlineStr">
         <is>
           <t>EXTRAVIO</t>
         </is>
@@ -1808,53 +1899,58 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="D25" s="8" t="n">
+      <c r="E25" s="8" t="n">
         <v>394</v>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Distribuidora Lima</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>T6U-711</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t>Jorge Quispe</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>DIESEL B5</t>
         </is>
       </c>
-      <c r="I25" s="10" t="n">
+      <c r="J25" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="J25" s="11" t="n">
+      <c r="K25" s="11" t="n">
         <v>16.8</v>
       </c>
-      <c r="K25" s="11">
-        <f>I25*J25</f>
-        <v/>
-      </c>
-      <c r="L25" s="8" t="inlineStr">
+      <c r="L25" s="11">
+        <f>J25*K25</f>
+        <v/>
+      </c>
+      <c r="M25" s="8" t="inlineStr">
         <is>
           <t>Luis G.</t>
         </is>
       </c>
-      <c r="M25" s="8" t="inlineStr">
+      <c r="N25" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N25" s="8" t="inlineStr">
+      <c r="O25" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1871,53 +1967,58 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="D26" s="8" t="n">
+      <c r="E26" s="8" t="n">
         <v>395</v>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>Minera Horizonte</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>V7X-551</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t>Alonso Ruiz</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
         <is>
           <t>PREMIUM</t>
         </is>
       </c>
-      <c r="I26" s="10" t="n">
+      <c r="J26" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="J26" s="11" t="n">
+      <c r="K26" s="11" t="n">
         <v>19.5</v>
       </c>
-      <c r="K26" s="11">
-        <f>I26*J26</f>
-        <v/>
-      </c>
-      <c r="L26" s="8" t="inlineStr">
+      <c r="L26" s="11">
+        <f>J26*K26</f>
+        <v/>
+      </c>
+      <c r="M26" s="8" t="inlineStr">
         <is>
           <t>Pedro M.</t>
         </is>
       </c>
-      <c r="M26" s="8" t="inlineStr">
+      <c r="N26" s="8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>
       </c>
-      <c r="N26" s="8" t="inlineStr">
+      <c r="O26" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1934,53 +2035,58 @@
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="D27" s="12" t="n">
+      <c r="E27" s="12" t="n">
         <v>396</v>
       </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G27" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H27" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I27" s="14" t="n">
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J27" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="15" t="n">
+      <c r="K27" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="K27" s="15">
-        <f>I27*J27</f>
-        <v/>
-      </c>
-      <c r="L27" s="12" t="inlineStr">
+      <c r="L27" s="15">
+        <f>J27*K27</f>
+        <v/>
+      </c>
+      <c r="M27" s="12" t="inlineStr">
         <is>
           <t>Mario S.</t>
         </is>
       </c>
-      <c r="M27" s="12" t="inlineStr">
+      <c r="N27" s="12" t="inlineStr">
         <is>
           <t>ANULADO</t>
         </is>
       </c>
-      <c r="N27" s="12" t="inlineStr">
+      <c r="O27" s="12" t="inlineStr">
         <is>
           <t>ERROR EN PLACA</t>
         </is>
@@ -1992,25 +2098,25 @@
           <t>TOTALES GENERALES:</t>
         </is>
       </c>
-      <c r="I28" s="17">
-        <f>SUM(I8:I27)</f>
-        <v/>
-      </c>
-      <c r="J28" s="18" t="n"/>
-      <c r="K28" s="19">
-        <f>SUM(K8:K27)</f>
-        <v/>
-      </c>
-      <c r="L28" s="18" t="n"/>
+      <c r="J28" s="17">
+        <f>SUM(J8:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="18" t="n"/>
+      <c r="L28" s="19">
+        <f>SUM(L8:L27)</f>
+        <v/>
+      </c>
       <c r="M28" s="18" t="n"/>
       <c r="N28" s="18" t="n"/>
+      <c r="O28" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="A28:I28"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A1:O1"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="M3:N3"/>
     <mergeCell ref="K4:L4"/>
@@ -2018,7 +2124,7 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="K3:L3"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="H3:I3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>